<commit_message>
WHSE Transaction Report: Completed the Report and apply the features to the report based on sir Elton's Instruction
</commit_message>
<xml_diff>
--- a/frontend/reports/notes_form/excluded_doc_no.xlsx
+++ b/frontend/reports/notes_form/excluded_doc_no.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-WAREHOUSE-PROGRAM-FRONTEND\frontend\reports\notes_form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F190777E-0596-43EE-B4DE-04B847A42A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF49E259-DA62-42B2-A3D9-6C85B0FBB9FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{91FDBA7B-8AD5-4C23-97C2-F2ED62C8AD71}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{91FDBA7B-8AD5-4C23-97C2-F2ED62C8AD71}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>